<commit_message>
Added final ppt for August | added few datasets
</commit_message>
<xml_diff>
--- a/Literature Review.xlsx
+++ b/Literature Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9412C44C-DE7B-4DBD-92BB-A5B1CE1F29F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFBE559-532C-411A-8651-739654723729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -60,21 +60,6 @@
     <t>Maximizing RAG efficiency: A comparative analysis of RAG methods</t>
   </si>
   <si>
-    <r>
-      <t>Cambridge University Press:  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF333333"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>30 October 2024</t>
-    </r>
-  </si>
-  <si>
     <t>EvaRAG: Evaluating Advanced RAG Techniques With Indexing and Distance Metrics</t>
   </si>
   <si>
@@ -106,13 +91,31 @@
   </si>
   <si>
     <t>Compares types of rag in Medical Field</t>
+  </si>
+  <si>
+    <t>Optimising clinical information extraction: a comparative study of retrieval-augmented generation techniques in clinical notes</t>
+  </si>
+  <si>
+    <t>Compares different retreival types in medical field</t>
+  </si>
+  <si>
+    <t>Evaluating Sparse and Dense Retrieval in Retrieval-Augmented Generation Systems: A Study</t>
+  </si>
+  <si>
+    <t>Association for computing machinery (ACM)</t>
+  </si>
+  <si>
+    <t>Hallucination across various RAG strategies</t>
+  </si>
+  <si>
+    <t>Cambridge University Press:  30 October 2024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,34 +140,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
-      <sz val="8"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF212529"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -172,18 +149,55 @@
     </font>
     <font>
       <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF212529"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF222222"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -214,31 +228,52 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -554,112 +589,181 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74087FDA-DCB0-42F6-A046-4BB743948387}">
-  <dimension ref="B6:F15"/>
+  <dimension ref="B3:F20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="85.44140625" customWidth="1"/>
-    <col min="4" max="4" width="36.44140625" customWidth="1"/>
+    <col min="4" max="4" width="44.109375" customWidth="1"/>
     <col min="5" max="5" width="32.33203125" customWidth="1"/>
     <col min="6" max="6" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:6" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="C6" s="1" t="s">
+    <row r="3" spans="2:6" ht="31.2" x14ac:dyDescent="0.6">
+      <c r="D3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="2:6" ht="21" x14ac:dyDescent="0.4">
+      <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="3">
+      <c r="B9" s="4">
         <v>1</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="11" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="6"/>
-      <c r="C10" s="7" t="s">
+      <c r="B10" s="6">
+        <v>2</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>10</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
     </row>
-    <row r="11" spans="2:6" ht="15" x14ac:dyDescent="0.35">
-      <c r="B11" s="6"/>
-      <c r="C11" s="6" t="s">
+    <row r="11" spans="2:6" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="B11" s="4">
+        <v>3</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>11</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>12</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
     </row>
-    <row r="12" spans="2:6" ht="15" x14ac:dyDescent="0.35">
-      <c r="B12" s="6"/>
-      <c r="C12" s="4" t="s">
+    <row r="12" spans="2:6" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="B12" s="6">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>12</v>
+      <c r="D12" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+      <c r="B13" s="4">
+        <v>5</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="6">
+        <v>6</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="4">
+        <v>7</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E14" t="s">
+      <c r="D15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="6">
+        <v>8</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
+      <c r="D16" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B17" s="4">
+        <v>9</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D15" t="s">
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="6">
         <v>10</v>
       </c>
-      <c r="E15" t="s">
-        <v>18</v>
-      </c>
+      <c r="C18" s="15"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C19" s="16"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C20" s="16"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -667,5 +771,6 @@
     <hyperlink ref="C12" r:id="rId2" display="https://aclanthology.org/2022.naacl-main.194.pdf" xr:uid="{69D0E201-038C-4594-A25F-23C3DA1E8BF8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added new research papers & updated the excel
</commit_message>
<xml_diff>
--- a/Literature Review.xlsx
+++ b/Literature Review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\rag-dissertation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFBE559-532C-411A-8651-739654723729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B974D350-CF24-45CB-BB43-749AA8DC607C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Subject</t>
   </si>
   <si>
-    <t>Outcome</t>
-  </si>
-  <si>
     <t>S.no.</t>
   </si>
   <si>
@@ -90,9 +87,6 @@
     <t>Compares different retreival types</t>
   </si>
   <si>
-    <t>Compares types of rag in Medical Field</t>
-  </si>
-  <si>
     <t>Optimising clinical information extraction: a comparative study of retrieval-augmented generation techniques in clinical notes</t>
   </si>
   <si>
@@ -105,17 +99,182 @@
     <t>Association for computing machinery (ACM)</t>
   </si>
   <si>
-    <t>Hallucination across various RAG strategies</t>
-  </si>
-  <si>
     <t>Cambridge University Press:  30 October 2024</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/abstract/document/11309712</t>
+  </si>
+  <si>
+    <t>https://www.cambridge.org/core/journals/natural-language-processing/article/maximizing-rag-efficiency-a-comparative-analysis-of-rag-methods/D7B259BCD35586E04358DF06006E0A85</t>
+  </si>
+  <si>
+    <t>Optimizing and comparing RAGs</t>
+  </si>
+  <si>
+    <t>Compares RAGs against Accuracy vs Efficiency</t>
+  </si>
+  <si>
+    <t>Compares different RAG eval frameworks</t>
+  </si>
+  <si>
+    <t>https://aclanthology.org/2025.xllm-1.14/</t>
+  </si>
+  <si>
+    <t>Provides new RAG for making system question type aware</t>
+  </si>
+  <si>
+    <t>https://aclanthology.org/2022.naacl-main.194/</t>
+  </si>
+  <si>
+    <t>Dissertation title - Hallucination across various RAG strategies</t>
+  </si>
+  <si>
+    <t>Ankit Mahto - 13454</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S1877050924021860</t>
+  </si>
+  <si>
+    <t>Survey compares different RAGs against Accuracy vs Efficiency</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1007/s00521-025-11666-9</t>
+  </si>
+  <si>
+    <t>Compares Rags on Medical Datasets</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/abstract/document/11245479</t>
+  </si>
+  <si>
+    <t>Compares different RAGs on different fields</t>
+  </si>
+  <si>
+    <t>Evaluating Retrieval-Augmented Generation Variants for Clinical Decision Support: Hallucination Mitigation and Secure On-Premises Deployment</t>
+  </si>
+  <si>
+    <t>MDPI</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2079-9292/14/21/4227</t>
+  </si>
+  <si>
+    <t>Compares Rags on Medical fields and optimizes to reduce hallucination during deployment</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S1532046426000778</t>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/10.1145/3708657.3708747</t>
+  </si>
+  <si>
+    <t>MEGA-RAG: a retrieval-augmented generation framework with multi-evidence guided answer refinement for mitigating hallucinations of LLMs in public health</t>
+  </si>
+  <si>
+    <t>Frontiers</t>
+  </si>
+  <si>
+    <t>MEGA Rag for public health domain</t>
+  </si>
+  <si>
+    <t>https://www.frontiersin.org/journals/public-health/articles/10.3389/fpubh.2025.1635381/full</t>
+  </si>
+  <si>
+    <t>Reducing Hallucinations and Trade-Offs in Responses in Generative AI Chatbots for Cancer Information: Development and Evaluation Study</t>
+  </si>
+  <si>
+    <t>International Journal on Engineering Artificial Intelligence Management, Decision Support, and Policies</t>
+  </si>
+  <si>
+    <t>Compares different RAGs on medical field</t>
+  </si>
+  <si>
+    <t>Retrieval-Augmented Generation (RAG) for Large Language Models: A Comprehensive Survey | International Journal on Engineering Artificial Intelligence Management, Decision Support, and Policies</t>
+  </si>
+  <si>
+    <t>Claim-Aware Scientific RAG: Evidence-First Retrieval and Abstention for Scientific Fact Responses on SciFact</t>
+  </si>
+  <si>
+    <t>Journal of Advanced Computing Systems (JACS)</t>
+  </si>
+  <si>
+    <t>Claim aware retrieval</t>
+  </si>
+  <si>
+    <t>https://scipublication.com/index.php/JACS/article/view/315</t>
+  </si>
+  <si>
+    <t>Retrieval Augmentation Reduces Factual Errors in Knowledge-Intensive Language Model Tasks</t>
+  </si>
+  <si>
+    <t>Computer Life</t>
+  </si>
+  <si>
+    <t>https://www.semanticscholar.org/paper/Retrieval-Augmentation-Reduces-Factual-Errors-in-Teng-Zhang/aef8626298e9cc4baf45000697e61626552fc2e4</t>
+  </si>
+  <si>
+    <t>Simple RAG with Eval</t>
+  </si>
+  <si>
+    <t>Hallucination in Retrieval-Augmented Generation is a Context Construction Problem: A Constraint-Driven Cross-Modal Framework</t>
+  </si>
+  <si>
+    <t>ACM</t>
+  </si>
+  <si>
+    <t>Constraint driven RAG framework for construction field</t>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/10.1145/3816713.3819507</t>
+  </si>
+  <si>
+    <t>Enhancing the Precision and Interpretability of Retrieval-Augmented Generation (RAG) in Legal Technology: A Survey</t>
+  </si>
+  <si>
+    <t>Compares RAGs against different metrics</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/10921633?denied=</t>
+  </si>
+  <si>
+    <t>Bridging Legal Knowledge and AI: Retrieval-Augmented Generation with Vector Stores, Knowledge Graphs, and Hierarchical Non-negative Matrix Factorization</t>
+  </si>
+  <si>
+    <t>RAG adaption for Legal Field</t>
+  </si>
+  <si>
+    <t>Bridging Legal Knowledge and AI: Retrieval-Augmented Generation with Vector Stores, Knowledge Graphs, and Hierarchical Non-negative Matrix Factorization | Proceedings of the Twentieth International Conference on Artificial Intelligence and Law</t>
+  </si>
+  <si>
+    <t>Towards Reliable Retrieval in RAG Systems for Large Legal Datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACL </t>
+  </si>
+  <si>
+    <t>Summary‑Augmented Chunking (SAC) for Legal documents</t>
+  </si>
+  <si>
+    <t>https://aclanthology.org/2025.nllp-1.3/</t>
+  </si>
+  <si>
+    <t>LegalGraphRAG: Multi-Agent Graph Retrieval-Augmented Generation for Reliable Legal Reasoning</t>
+  </si>
+  <si>
+    <t>LEGALGRAPH RAG for legal field</t>
+  </si>
+  <si>
+    <t>https://aclanthology.org/2026.acl-long.1738/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,14 +301,6 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -185,8 +336,49 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF172B4D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF212121"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,6 +388,42 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -228,52 +456,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -290,6 +564,615 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>27584</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="582706" cy="291352"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="TextBox 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2ED19ED4-A8B9-4CA0-88E2-042262DE8E21}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1210235" y="1954996"/>
+          <a:ext cx="582706" cy="291352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent5">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>509867</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>145676</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3569074" cy="329711"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="TextBox 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{177705F6-AF94-4E4A-8084-FD15556F5280}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1720102" y="1882588"/>
+          <a:ext cx="3569074" cy="329711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1"/>
+            <a:t>Closest to current dissertation topic</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>4347882</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>27585</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="582706" cy="291352"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="TextBox 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3524C272-9DE8-45C3-AFC0-6E5D980F32B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5558117" y="1954997"/>
+          <a:ext cx="582706" cy="291352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>4857749</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>145677</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3569074" cy="329711"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="TextBox 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CBB883A7-E178-4025-A5A9-BB166E9B7CB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6067984" y="1882589"/>
+          <a:ext cx="3569074" cy="329711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1"/>
+            <a:t>Architecture</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1" baseline="0"/>
+            <a:t> comparisons</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1800" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1400736</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9654</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="582706" cy="291352"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="TextBox 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F091DE7-4DBE-4FDA-B286-89C615471187}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8975912" y="1937066"/>
+          <a:ext cx="582706" cy="291352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent6">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1910603</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>127746</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3569074" cy="329711"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="TextBox 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6941BC8E-FE65-41BC-A492-4B0785F118CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9485779" y="1864658"/>
+          <a:ext cx="3569074" cy="329711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1"/>
+            <a:t>Comparisons</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1" baseline="0"/>
+            <a:t> in medical field</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1800" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2191870</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>162054</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="582706" cy="291352"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="TextBox 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2F62BA80-C937-48A6-ABFB-E88BDB886742}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12714194" y="1898966"/>
+          <a:ext cx="582706" cy="291352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2701737</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>89646</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3569074" cy="329711"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="TextBox 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA432220-2433-4677-99E9-B85F65AE734A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13224061" y="1826558"/>
+          <a:ext cx="3569074" cy="329711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1"/>
+            <a:t>Legal related</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4641476</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>157572</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="582706" cy="291352"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="TextBox 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C0DB847-8CDF-47D0-AC17-831B3C31FC0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15163800" y="1894484"/>
+          <a:ext cx="582706" cy="291352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg2">
+            <a:lumMod val="90000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>5151343</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>85164</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3569074" cy="329711"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="TextBox 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6649402B-C006-4D35-8E8E-1972FD421F83}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15673667" y="1822076"/>
+          <a:ext cx="3569074" cy="329711"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1"/>
+            <a:t>Less</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1800" b="1" baseline="0"/>
+            <a:t> relavant</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1800" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -589,188 +1472,398 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74087FDA-DCB0-42F6-A046-4BB743948387}">
-  <dimension ref="B3:F20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B3:F32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="85.44140625" customWidth="1"/>
-    <col min="4" max="4" width="44.109375" customWidth="1"/>
-    <col min="5" max="5" width="32.33203125" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="95.42578125" customWidth="1"/>
+    <col min="4" max="4" width="44.140625" customWidth="1"/>
+    <col min="5" max="5" width="89.85546875" customWidth="1"/>
+    <col min="6" max="6" width="44.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:6" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:6" ht="31.5" x14ac:dyDescent="0.5">
       <c r="D3" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="C6" s="32" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:6" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="B13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="6">
+        <v>2</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="29" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="B8" s="3" t="s">
+    <row r="16" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8">
+        <v>3</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="6">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C17" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="29" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="8">
+        <v>5</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="6">
         <v>6</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="4">
-        <v>1</v>
-      </c>
-      <c r="C9" s="11" t="s">
+      <c r="C19" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="8">
         <v>7</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="6">
-        <v>2</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="C20" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E20" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="29" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B21" s="12">
+        <v>8</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="14">
         <v>9</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" spans="2:6" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B11" s="4">
-        <v>3</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="C22" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B23" s="12">
         <v>10</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="C23" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" s="30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B24" s="12">
         <v>11</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-    </row>
-    <row r="12" spans="2:6" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B12" s="6">
-        <v>4</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="4">
-        <v>5</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="C24" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E24" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="18">
+        <v>12</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" s="31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="18">
         <v>13</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="6">
-        <v>6</v>
-      </c>
-      <c r="C14" s="12" t="s">
+      <c r="C26" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F26" s="31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B27" s="18">
         <v>14</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="C27" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F27" s="31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B28" s="19">
         <v>15</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="C28" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="B29" s="19">
+        <v>16</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="19">
+        <v>17</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="19">
         <v>18</v>
       </c>
-      <c r="F14" s="6"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="4">
-        <v>7</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="C31" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B32" s="19">
+        <v>19</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="6">
-        <v>8</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="6"/>
-    </row>
-    <row r="17" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="4">
-        <v>9</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="6"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="6">
+      <c r="D32" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C19" s="16"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C20" s="16"/>
+      <c r="E32" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C9" r:id="rId1" display="https://aclanthology.org/2022.naacl-main.194.pdf" xr:uid="{68E5C6A5-EDD3-4584-9F9D-6426C53B75D7}"/>
-    <hyperlink ref="C12" r:id="rId2" display="https://aclanthology.org/2022.naacl-main.194.pdf" xr:uid="{69D0E201-038C-4594-A25F-23C3DA1E8BF8}"/>
+    <hyperlink ref="F28" r:id="rId1" xr:uid="{B72BA10E-195C-4795-8410-88E6B771479E}"/>
+    <hyperlink ref="F27" r:id="rId2" display="https://dl.acm.org/doi/10.1145/3769126.3769215" xr:uid="{519F6847-1D7B-4426-A60A-6D4F4AB956C9}"/>
+    <hyperlink ref="F32" r:id="rId3" xr:uid="{E68171B4-3071-4FD9-B15A-6F5BE20AF5DE}"/>
+    <hyperlink ref="F23" r:id="rId4" display="https://submissions.adroidjournals.com/index.php/ijaimd/article/view/233" xr:uid="{BDD37FC8-C1B4-46B0-B984-AC20EBCC3CE9}"/>
+    <hyperlink ref="F17" r:id="rId5" xr:uid="{AD9D2951-BEE1-4DC2-9403-9C3A71810B3A}"/>
+    <hyperlink ref="F15" r:id="rId6" xr:uid="{A1D44CA5-5B75-45A1-B02F-7445AD8D9836}"/>
+    <hyperlink ref="F16" r:id="rId7" xr:uid="{1D7D364A-4EB5-4994-A83D-E2EA55357BA9}"/>
+    <hyperlink ref="F14" r:id="rId8" xr:uid="{F8D7FD10-FC41-4FCA-89F5-71C096C077D5}"/>
+    <hyperlink ref="F18" r:id="rId9" xr:uid="{181AB44D-A5F5-4541-A1D7-EEBBD8144E20}"/>
+    <hyperlink ref="F20" r:id="rId10" xr:uid="{9D431151-8205-48B5-B777-C0F9EE704D5C}"/>
+    <hyperlink ref="F19" r:id="rId11" xr:uid="{22C9E69A-64AF-4FF8-B485-CB65221CAE64}"/>
+    <hyperlink ref="F21" r:id="rId12" xr:uid="{1CF964EC-CB9C-467E-962A-D95FE364740E}"/>
+    <hyperlink ref="F22" r:id="rId13" xr:uid="{66C78296-53DE-4B9D-9119-C5A2A43FC383}"/>
+    <hyperlink ref="F24" r:id="rId14" xr:uid="{085DD53A-7B1B-4F53-B67D-5D20BF06C8FB}"/>
+    <hyperlink ref="F26" r:id="rId15" xr:uid="{664BB049-AF7C-4CBF-8DE7-F0EE22581E1F}"/>
+    <hyperlink ref="F25" r:id="rId16" xr:uid="{FF241946-5ACD-4BC8-BFE7-ED1B29E79B07}"/>
+    <hyperlink ref="F29" r:id="rId17" xr:uid="{BC650767-95BB-4E6C-A352-66EA0C6382B6}"/>
+    <hyperlink ref="F31" r:id="rId18" xr:uid="{EE7FC2B8-58DA-4DC2-A367-F2E69D94E67D}"/>
+    <hyperlink ref="F30" r:id="rId19" xr:uid="{C3301100-1845-4B84-8BBF-A20F72300684}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
+  <drawing r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
made naive rag work | optimized a bit
</commit_message>
<xml_diff>
--- a/Literature Review.xlsx
+++ b/Literature Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B974D350-CF24-45CB-BB43-749AA8DC607C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FC3B9D-E33E-4EBF-8FFB-E530C66EDE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -138,9 +138,6 @@
     <t>https://www.sciencedirect.com/science/article/pii/S1877050924021860</t>
   </si>
   <si>
-    <t>Survey compares different RAGs against Accuracy vs Efficiency</t>
-  </si>
-  <si>
     <t>https://link.springer.com/article/10.1007/s00521-025-11666-9</t>
   </si>
   <si>
@@ -268,6 +265,12 @@
   </si>
   <si>
     <t>https://aclanthology.org/2026.acl-long.1738/</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Survey compares different RAGs against Accuracy vs Efficiency across various fields</t>
   </si>
 </sst>
 </file>
@@ -456,7 +459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -548,6 +551,11 @@
       <alignment horizontal="fill" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1472,7 +1480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74087FDA-DCB0-42F6-A046-4BB743948387}">
-  <dimension ref="B3:F32"/>
+  <dimension ref="B3:G32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="95.42578125" customWidth="1"/>
@@ -1481,26 +1489,26 @@
     <col min="6" max="6" width="44.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:6" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:7" ht="31.5" x14ac:dyDescent="0.5">
       <c r="D3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C4" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:7" ht="26.25" x14ac:dyDescent="0.4">
       <c r="C6" s="32" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:6" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:7" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1516,8 +1524,11 @@
       <c r="F13" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="33" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
         <v>1</v>
       </c>
@@ -1528,13 +1539,14 @@
         <v>8</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="G14" s="34"/>
+    </row>
+    <row r="15" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
         <v>2</v>
       </c>
@@ -1550,8 +1562,9 @@
       <c r="F15" s="29" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G15" s="34"/>
+    </row>
+    <row r="16" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="8">
         <v>3</v>
       </c>
@@ -1567,8 +1580,9 @@
       <c r="F16" s="29" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="2:6" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="G16" s="34"/>
+    </row>
+    <row r="17" spans="2:7" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
         <v>4</v>
       </c>
@@ -1584,8 +1598,9 @@
       <c r="F17" s="29" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="18" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="34"/>
+    </row>
+    <row r="18" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="8">
         <v>5</v>
       </c>
@@ -1596,13 +1611,14 @@
         <v>12</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="F18" s="29" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="34"/>
+    </row>
+    <row r="19" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
         <v>6</v>
       </c>
@@ -1616,44 +1632,47 @@
         <v>16</v>
       </c>
       <c r="F19" s="29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="G19" s="34"/>
+    </row>
+    <row r="20" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="8">
         <v>7</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="29" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G20" s="34"/>
+    </row>
+    <row r="21" spans="2:7" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B21" s="12">
         <v>8</v>
       </c>
       <c r="C21" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="E21" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="F21" s="30" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G21" s="34"/>
+    </row>
+    <row r="22" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="14">
         <v>9</v>
       </c>
@@ -1664,30 +1683,32 @@
         <v>14</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="G22" s="34"/>
+    </row>
+    <row r="23" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B23" s="12">
         <v>10</v>
       </c>
       <c r="C23" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="E23" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="F23" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="30" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="35"/>
+    </row>
+    <row r="24" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B24" s="12">
         <v>11</v>
       </c>
@@ -1701,129 +1722,137 @@
         <v>18</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="G24" s="35"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="18">
         <v>12</v>
       </c>
       <c r="C25" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="E25" s="24" t="s">
+      <c r="F25" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="F25" s="31" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="35"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="18">
         <v>13</v>
       </c>
       <c r="C26" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="E26" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="31" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G26" s="35"/>
+    </row>
+    <row r="27" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B27" s="18">
         <v>14</v>
       </c>
       <c r="C27" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E27" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="F27" s="31" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G27" s="35"/>
+    </row>
+    <row r="28" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B28" s="19">
         <v>15</v>
       </c>
       <c r="C28" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="E28" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="21" t="s">
+      <c r="F28" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="F28" s="27" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G28" s="35"/>
+    </row>
+    <row r="29" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B29" s="19">
         <v>16</v>
       </c>
       <c r="C29" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="E29" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="F29" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="F29" s="27" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="35"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="19">
         <v>17</v>
       </c>
       <c r="C30" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="E30" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="E30" s="21" t="s">
+      <c r="F30" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="F30" s="27" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="35"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="19">
         <v>18</v>
       </c>
       <c r="C31" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="E31" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F31" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="E31" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="F31" s="27" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="G31" s="35"/>
+    </row>
+    <row r="32" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B32" s="19">
         <v>19</v>
       </c>
@@ -1839,6 +1868,7 @@
       <c r="F32" s="27" t="s">
         <v>28</v>
       </c>
+      <c r="G32" s="35"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Finished Naive RAG| Finalized for code for presentation | created final ppt | updated monthly report docs
</commit_message>
<xml_diff>
--- a/Literature Review.xlsx
+++ b/Literature Review.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Projects\rag-dissertation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FC3B9D-E33E-4EBF-8FFB-E530C66EDE71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CF8342-F718-4E1D-A7B8-4E9AC6DE33BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="79">
   <si>
     <t>LITERATURE REVIEW</t>
   </si>
@@ -459,7 +459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -554,8 +554,36 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="fill"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1481,34 +1509,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74087FDA-DCB0-42F6-A046-4BB743948387}">
   <dimension ref="B3:G32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="95.42578125" customWidth="1"/>
-    <col min="4" max="4" width="44.140625" customWidth="1"/>
-    <col min="5" max="5" width="89.85546875" customWidth="1"/>
-    <col min="6" max="6" width="44.140625" customWidth="1"/>
+    <col min="3" max="3" width="95.44140625" customWidth="1"/>
+    <col min="4" max="4" width="44.109375" customWidth="1"/>
+    <col min="5" max="5" width="89.88671875" customWidth="1"/>
+    <col min="6" max="6" width="44.109375" customWidth="1"/>
+    <col min="7" max="7" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:7" ht="31.2" x14ac:dyDescent="0.6">
       <c r="D3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="18" x14ac:dyDescent="0.35">
       <c r="C4" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:7" ht="25.8" x14ac:dyDescent="0.5">
       <c r="C6" s="32" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:7" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="2:7" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1528,7 +1557,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5">
         <v>1</v>
       </c>
@@ -1544,9 +1573,11 @@
       <c r="F14" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="34"/>
-    </row>
-    <row r="15" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="6">
         <v>2</v>
       </c>
@@ -1562,9 +1593,11 @@
       <c r="F15" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="34"/>
-    </row>
-    <row r="16" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G15" s="39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="8">
         <v>3</v>
       </c>
@@ -1580,9 +1613,11 @@
       <c r="F16" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="G16" s="34"/>
-    </row>
-    <row r="17" spans="2:7" s="4" customFormat="1" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="G16" s="29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" s="4" customFormat="1" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B17" s="6">
         <v>4</v>
       </c>
@@ -1598,9 +1633,11 @@
       <c r="F17" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="G17" s="34"/>
-    </row>
-    <row r="18" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="34" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="8">
         <v>5</v>
       </c>
@@ -1616,9 +1653,11 @@
       <c r="F18" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="G18" s="34"/>
-    </row>
-    <row r="19" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="29" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6">
         <v>6</v>
       </c>
@@ -1634,9 +1673,11 @@
       <c r="F19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="G19" s="34"/>
-    </row>
-    <row r="20" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G19" s="35" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B20" s="8">
         <v>7</v>
       </c>
@@ -1652,9 +1693,11 @@
       <c r="F20" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="G20" s="34"/>
-    </row>
-    <row r="21" spans="2:7" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G20" s="43" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" s="4" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B21" s="12">
         <v>8</v>
       </c>
@@ -1670,9 +1713,11 @@
       <c r="F21" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="G21" s="34"/>
-    </row>
-    <row r="22" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G21" s="42" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B22" s="14">
         <v>9</v>
       </c>
@@ -1688,9 +1733,11 @@
       <c r="F22" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="34"/>
-    </row>
-    <row r="23" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G22" s="30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B23" s="12">
         <v>10</v>
       </c>
@@ -1706,9 +1753,11 @@
       <c r="F23" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="35"/>
-    </row>
-    <row r="24" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B24" s="12">
         <v>11</v>
       </c>
@@ -1724,9 +1773,11 @@
       <c r="F24" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="G24" s="35"/>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B25" s="18">
         <v>12</v>
       </c>
@@ -1742,9 +1793,11 @@
       <c r="F25" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="G25" s="35"/>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G25" s="40" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B26" s="18">
         <v>13</v>
       </c>
@@ -1760,9 +1813,11 @@
       <c r="F26" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="G26" s="35"/>
-    </row>
-    <row r="27" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G26" s="40" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B27" s="18">
         <v>14</v>
       </c>
@@ -1778,9 +1833,11 @@
       <c r="F27" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="G27" s="35"/>
-    </row>
-    <row r="28" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G27" s="37" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B28" s="19">
         <v>15</v>
       </c>
@@ -1796,9 +1853,11 @@
       <c r="F28" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="G28" s="35"/>
-    </row>
-    <row r="29" spans="2:7" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G28" s="38" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B29" s="19">
         <v>16</v>
       </c>
@@ -1814,9 +1873,11 @@
       <c r="F29" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="G29" s="35"/>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G29" s="41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" s="19">
         <v>17</v>
       </c>
@@ -1832,9 +1893,11 @@
       <c r="F30" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="G30" s="35"/>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G30" s="27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="19">
         <v>18</v>
       </c>
@@ -1850,9 +1913,11 @@
       <c r="F31" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="G31" s="35"/>
-    </row>
-    <row r="32" spans="2:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="G31" s="27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="B32" s="19">
         <v>19</v>
       </c>
@@ -1868,7 +1933,9 @@
       <c r="F32" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="G32" s="35"/>
+      <c r="G32" s="27" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1891,9 +1958,23 @@
     <hyperlink ref="F29" r:id="rId17" xr:uid="{BC650767-95BB-4E6C-A352-66EA0C6382B6}"/>
     <hyperlink ref="F31" r:id="rId18" xr:uid="{EE7FC2B8-58DA-4DC2-A367-F2E69D94E67D}"/>
     <hyperlink ref="F30" r:id="rId19" xr:uid="{C3301100-1845-4B84-8BBF-A20F72300684}"/>
+    <hyperlink ref="G14" r:id="rId20" xr:uid="{8D88101D-7C46-4B4C-9949-A6DBD99222E5}"/>
+    <hyperlink ref="G15" r:id="rId21" xr:uid="{78A5001E-405F-409B-B470-973DEE3D38CD}"/>
+    <hyperlink ref="G16" r:id="rId22" xr:uid="{2835E438-A848-4EDB-917F-6015DB2BAD8D}"/>
+    <hyperlink ref="G18" r:id="rId23" xr:uid="{BB27E631-DA69-4903-B478-4972BE708DEE}"/>
+    <hyperlink ref="G32" r:id="rId24" xr:uid="{FB02735D-6D36-4A6D-AC53-38B5D056C8EA}"/>
+    <hyperlink ref="G26" r:id="rId25" xr:uid="{BD268B87-26D3-43C7-B5D8-19E1A93A38EE}"/>
+    <hyperlink ref="G29" r:id="rId26" xr:uid="{38A0110B-5BE0-4B19-92C2-AE10EE26FE76}"/>
+    <hyperlink ref="G24" r:id="rId27" xr:uid="{E76FE7BA-21A9-4C6E-89C1-1B21B0072E41}"/>
+    <hyperlink ref="G25" r:id="rId28" xr:uid="{29AC8029-1F97-4235-AA0D-CB3EF060377C}"/>
+    <hyperlink ref="G21" r:id="rId29" xr:uid="{81E9BEBC-7364-4245-8CDB-91EA87F24E0A}"/>
+    <hyperlink ref="G30" r:id="rId30" xr:uid="{5561AB18-DCED-4134-816F-31FBB95B1C9F}"/>
+    <hyperlink ref="G31" r:id="rId31" xr:uid="{6561F8EB-D24A-4389-8F60-1F81DDA14483}"/>
+    <hyperlink ref="G22" r:id="rId32" xr:uid="{4A48ADCB-7472-400E-9D7F-45C3E4B93026}"/>
+    <hyperlink ref="G20" r:id="rId33" xr:uid="{935A5B9B-3F16-4040-A2BD-A875F391627B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId20"/>
-  <drawing r:id="rId21"/>
+  <pageSetup orientation="portrait" r:id="rId34"/>
+  <drawing r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>